<commit_message>
feat(masterdata): TbGameMode에 scene_path 추가
게임 모드가 자기 게임 씬을 가리키게 한다. 지금까지 씬 이름은 유니티 코드에
상수로 박혀 있어 gameModeId가 아무것도 결정하지 못했다.

##group을 c,s로 지정해 유니티(클라·서버)에만 들어가고 matchmaking 서버
생성물에는 빠지게 했다 — 매치메이커는 씬 경로를 몰라도 되고, id/code/
minPlayers/maxPlayers만 읽으면 된다. (빈 칸은 "그룹 필터 없음 = 모든
타깃에 포함"이라 오히려 matchmaking에도 새 나갔던 걸 확인 후 c,s로 수정)

fix(masterdata): gen.sh가 지운 유니티 .meta를 자동 복원

Luban이 -t client/-t server 생성 전에 Scripts/MasterData,
StreamingAssets/MasterData를 rm -rf로 통째로 지우는데, 유니티가 만든
.meta 파일은 Luban이 다시 만들어주지 않는다. 그래서 매번 생성할 때마다
git이 추적하던 .meta가 "삭제됨"으로 남았다(이번에 82개). rm -rf 직후
지워진 .meta만 골라 git에서 원래대로 되돌리는 단계를 client/server 각각에
추가했다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#GameMode.xlsx
+++ b/table/Datas/#GameMode.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,11 @@
           <t>max_players</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>scene_path</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -489,6 +494,11 @@
           <t>int</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -496,8 +506,6 @@
           <t>##group</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>c</t>
@@ -508,8 +516,11 @@
           <t>c</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>c,s</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -545,6 +556,11 @@
       <c r="G4" t="inlineStr">
         <is>
           <t>max_players</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scene_path</t>
         </is>
       </c>
     </row>
@@ -562,12 +578,16 @@
           <t>플랩왕</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
         <v>2</v>
       </c>
       <c r="G5" t="n">
         <v>8</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Assets/Scenes/FlapWang.unity</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -584,7 +604,6 @@
           <t>닷지볼</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
         <v>2</v>
       </c>
@@ -606,7 +625,6 @@
           <t>관찰자 피하기</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
         <v>2</v>
       </c>
@@ -628,7 +646,6 @@
           <t>기억력 게임</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
         <v>2</v>
       </c>
@@ -650,7 +667,6 @@
           <t>타겟 슈팅</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
feat(masterdata): FlappyRace 게임 모드와 맵을 추가한다
TbGameMode id=6, TbMap id=2. 큐의 allowed_game_mode_ids에도 6을 넣는다 —
안 넣으면 매치메이킹 서버가 티켓을 INVALID_GAME_MODE로 되돌린다.

min_players를 1로 둔 건 혼자 접속해도 매칭이 성사돼야 이 축이 실제로
갈라지는지 확인할 수 있어서다. 실제 인원 요건은 종료·순위 슬라이스에서 정한다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#GameMode.xlsx
+++ b/table/Datas/#GameMode.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -674,6 +674,43 @@
         <v>8</v>
       </c>
     </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FlappyRace</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>플래피 레이스</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>날개짓으로 코스를 통과해 결승선에 먼저 닿는 레이스</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Assets/Scenes/FlappyRace.unity</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>